<commit_message>
Update news list: 2026-05-26
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -890,6 +890,72 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2024.10.16 11:03</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>영업 취소 결정 전 ‘영업자 사정’ 우선 살핀다</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=28462</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2024.10.10 17:59</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>배달플랫폼 수수료 부담완화 위한 상생방안 마련</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=28459</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2024.10.10 14:48</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>스마트오더 주류 주문 시 신분증확인 절차 미흡해</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=28457</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-06-02
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -956,6 +956,50 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026.06.01 15:55</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>'외식 환경 개선' 나주시, 식품안심업소 지정 확대·컨설팅 지원</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30220</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026.05.29 10:47</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>무료로 배우고 취업까지…중구, 외식업 실무 전문가 양성과정 교육생 모집</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30222</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-06-18
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1000,6 +1000,28 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026.06.17 14:13</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>(사)한국외식업중앙회 경북지회 경산시지부, 사랑의 음식나누기 행사 개최</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30267</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-06-19
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1022,6 +1022,28 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026.06.18 16:26</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>충남도, ‘외국인 친화 음식점’ 100곳 공개 모집</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30280</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-06-23
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1044,6 +1044,28 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026.06.22 16:28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>의령군-외식업중앙회 의령군지부, 식중독 예방 거리 캠페인</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30292</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-07
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1066,6 +1066,28 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026.07.06 14:05</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>정읍시, 소상공인 카드 수수료 최대 30만원 지원… 6일부터 접수</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30317</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-09
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1088,6 +1088,72 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026.07.08 09:29</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>경남도 박완수 지사 “외식업계 현장 목소리 반영해 경쟁력 강화 지원”</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30334</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026.07.08 09:28</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>창녕군, 산토끼밥상 활성화 위해 ‘군청·이방면 외식의 날’ 운영</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30332</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026.07.08 09:28</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>장성군, 외식업소 매출 살릴 ‘경영 처방전’ 제공</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30330</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-10
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1154,6 +1154,28 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026.07.09 16:22</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>포천시농업재단-외식업중앙회, 지역 농산물 활용 조리실무교육 성료</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30340</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-13
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1176,6 +1176,28 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026.07.13 15:44</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>식약처, 삼계탕·냉면·치킨 배달음식점 등 3천700여 곳 위생관리 강화</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30353</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-16
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1198,6 +1198,72 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026.07.15 10:27</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>서초구, 외식업주 위한 블랙컨슈머 대응체계 구축</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30386</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026.07.15 09:39</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>AI·빅데이터가 콕 집었다…경북문화관광公, '경북 디저트 지도' 공개</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30379</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026.07.15 09:07</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>음성군, 일반음식점 주방환경개선 지원사업 추진</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30382</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-20
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1264,6 +1264,28 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026.07.20 13:16</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>충장축제, 시민 참여 프로그램 참가자 모집</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30413</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-21
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1286,6 +1286,72 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026.07.21 15:07</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>파주시, ‘2026년도 외식업체 전문경영 컨설팅’ 참여 업소 모집</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30431</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026.07.21 10:56</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>거제시, 식품 관련 공무원 사칭사기 주의</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30424</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026.07.21 10:13</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>인제군, 소상공인 배달비 부담에 ‘든든한 우산’... 먹깨비 배달비 지원 3천원으로 확대</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30420</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-22
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1352,6 +1352,28 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026.07.22 14:04</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>보성군, 일반음식점 영업주 위생·친절교육 실시</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30449</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-23
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1374,6 +1374,28 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026.07.23 09:56</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>구미시, 「K-외식산업 기반구축 지원」 참여업소 모집</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30457</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-25
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1396,6 +1396,28 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026.07.24 09:35</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>예금토큰, 카드처럼 쓴다…소상공인 수수료 부담 던다</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30482</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-29
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1418,6 +1418,50 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026.07.29 13:45</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>예산군, 별점 5개로 더 쉽게 확인하는 ‘식품안심업소’</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30522</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026.07.29 13:38</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>"20만원 내면 40만원 휴가비"…정부, 알뜰 여름휴가 서비스 공개</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30518</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-07-31
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1462,6 +1462,28 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026.07.31 10:04</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>"남은 소스, 배달용기 어쩌나"…10월부터 식당 위생기준 강화</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30535</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-04
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1484,6 +1484,50 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026.08.03 10:36</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>영주시, 외식업 경쟁력 강화를 위한 디지털 전환 사업 참여업체 모집</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30548</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026.08.03 10:32</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>현장 중심, 맞춤형 지원의 시작… 남양주시, 소상공인 ‘든든지원단’ 운영 개시</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30544</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-05
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1550,6 +1550,94 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026.08.05 14:09</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>‘시민혜택 올리고, 소상공인 매출 늘리고’… 남양주시, 온누리상품권 사용처 확대</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30589</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026.08.05 12:50</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>동작구, 소상공인 휴업손실보상보험 지원대상 확대…거주요건 폐지·영업기간 기준 완화</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30583</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026.08.05 11:20</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>익산시, 청년 외식 창업 디딤돌 '공유주방' 참여자 모집</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30575</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026.08.05 08:56</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>마포구, 중소기업·소상공인에 20억 융자 지원…11일까지 신청 접수</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30585</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-07
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1638,6 +1638,28 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026.08.06 14:12</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>나주 대표 맛집 브랜드 ‘나주밥상’ 49곳으로 확대</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30598</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-10
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1660,6 +1660,28 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026.08.10 11:09</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>연매출 4억원 이하 식당, 부가세 우대 공제 2년 연장</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30610</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-13
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1682,6 +1682,28 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026.08.13 14:30</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>예천군 외식업소 친절교육 수료식… 현장 서비스 역량 높여</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30621</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-18
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1704,6 +1704,28 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026.08.18 14:44</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>인천시, 반려동물 동반 출입 음식점에 지원물품 배부…</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30629</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-20
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1726,6 +1726,72 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026.08.20 15:32</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>경주시, 아동친화음식점‘웰컴키즈존’50곳 추가 모집</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30643</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026.08.20 15:31</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>남은 음식 버리지 말고 포장하세요...삼척시 포장용기 지원</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30641</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026.08.20 15:30</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>제주시, 음식물류 폐기물 다량배출사업자 지도·점검</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30639</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-24
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1792,6 +1792,28 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026.08.21 20:03</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>'시민 안전 외식' 영주시, 식품안심업소 모집</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30659</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-08-29
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1814,6 +1814,94 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026.08.27 15:35</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>동해시, 배달음식점·기차역 주변 업소 위생 점검 ‘먹거리 안전망’ 강화</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30681</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026.08.27 15:31</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>당진시, 도민체전 대비 식품․공중 위생 집중 점검</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30677</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026.08.27 15:30</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>남해군, ‘혼자와도 좋은식당’ 모집</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30675</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026.08.27 15:28</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>울산시-경남은행-울산신보 지역 소상공인에 500억 원 금융 지원</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30673</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-01
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1902,6 +1902,28 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026.08.24 22:07</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>경주시, 식품안심업소 영업장 내부 청소비 지원…최대 50만원</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30683</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-02
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1924,6 +1924,50 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026.09.01 16:01</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>음식점 바가지요금 처벌 강화, 적발 시 영업정지</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30707</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026.09.01 09:25</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>보성군, ‘2026 보성 미식 아카데미’ 참여자 모집</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30698</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-03
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1968,6 +1968,28 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026.09.02 10:10</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>'블랙컨슈머 대응 특강'…서초구, 외식업주 대상 실전 교육 실시</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30717</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-04
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1990,6 +1990,28 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026.09.03 17:03</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>창원특례시, 지역상생 문화장터 「도계부부 달빛야시장」 9월 개장</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30736</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-05
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2012,6 +2012,28 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026.09.04 11:20</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>춘천시, 관광지 음식점 1회용품 사용 줄이기 점검</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30746</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>